<commit_message>
add after 1j pertubation
</commit_message>
<xml_diff>
--- a/docs/cadrage/product-backlog.xlsx
+++ b/docs/cadrage/product-backlog.xlsx
@@ -8,24 +8,39 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsiba\Documents\cours\Master IA\apocalIPSSI\IPSSI_APOCAL_KIT_GR_28\docs\cadrage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61369215-FDE3-4C71-9503-D381E727B262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A47408-93F1-45EE-BE82-4D3FA25DE6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" r:id="rId1"/>
     <sheet name="Identification" sheetId="2" r:id="rId2"/>
     <sheet name="Epics" sheetId="3" r:id="rId3"/>
     <sheet name="Backlog" sheetId="4" r:id="rId4"/>
-    <sheet name="DoR &amp; DoD" sheetId="5" r:id="rId5"/>
-    <sheet name="Auto-évaluation" sheetId="6" r:id="rId6"/>
+    <sheet name="Epics-post-1j" sheetId="7" r:id="rId5"/>
+    <sheet name="Backlog-post-1j" sheetId="8" r:id="rId6"/>
+    <sheet name="DoR &amp; DoD" sheetId="5" r:id="rId7"/>
+    <sheet name="Auto-évaluation" sheetId="6" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="641" uniqueCount="215">
   <si>
     <t>A</t>
   </si>
@@ -663,12 +678,80 @@
   <si>
     <t>S8</t>
   </si>
+  <si>
+    <t>US-21</t>
+  </si>
+  <si>
+    <t>US-22</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignant·e, je veux pouvoir consulter le resultat d'un etudiant</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignant·e, je veux pouvoir identifer un etudiant decrocheurs</t>
+  </si>
+  <si>
+    <t>G: Liste des etudiants de l'enseignante
+W: la page se charge
+T: liste des etudiants triés par (note,date) desc, avec nom/date/score/…..</t>
+  </si>
+  <si>
+    <t>G: donnée statisqtique de l'etudiant sur [X] mois
+W: consulte
+T: met en evidance les lacunes et par matiere et les notes</t>
+  </si>
+  <si>
+    <t>US-23</t>
+  </si>
+  <si>
+    <t>US-24</t>
+  </si>
+  <si>
+    <t>US-25</t>
+  </si>
+  <si>
+    <t>US-26</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignant·e je veux un dashboard de progression pour suivre mes etudiants.</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignant·e je veux des filters pour mieux ciblé mes etudiants.</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignant·e je veux ouvoir envoyer des coneille à mes etudaints sur leurs lacunes.</t>
+  </si>
+  <si>
+    <t>En tant qu'enseignant·e je veux un espace numerique pour moi.</t>
+  </si>
+  <si>
+    <t>26 stories · 161 SP scope total · à arbitrer contre vélocité cible ~56 SP</t>
+  </si>
+  <si>
+    <t>1 critère type :   page /dashboard avec graphique en barres score / chap.</t>
+  </si>
+  <si>
+    <t>1 critère type :   zone de commentaire a tribuer à l'enseignant·e</t>
+  </si>
+  <si>
+    <t>1 critère type :   page /Liste des etudiants affilier</t>
+  </si>
+  <si>
+    <t>1 critère type :   filtre sur les liste etudiante</t>
+  </si>
+  <si>
+    <t>US-12, US-17,US-24</t>
+  </si>
+  <si>
+    <t>US-06, US-11, US-16,US-21
+US-22,US-23,US-25,US-26</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -838,6 +921,33 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF1E1B4B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF475569"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1E1B4B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1E1B4B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -931,7 +1041,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1019,8 +1129,24 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1616,8 +1742,7 @@
   <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="8" style="41" customWidth="1"/>
+    <col min="1" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="9" style="24" customWidth="1"/>
@@ -1642,7 +1767,7 @@
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="9" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1650,7 +1775,7 @@
       <c r="A5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="9" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1658,7 +1783,7 @@
       <c r="A6" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="9" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1666,7 +1791,7 @@
       <c r="A7" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="42" t="s">
+      <c r="B7" s="9" t="s">
         <v>58</v>
       </c>
     </row>
@@ -2430,6 +2555,1188 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FC90CA6-3212-4A11-8B04-F3F237D99480}">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A6" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="14">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="14">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="14">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>214</v>
+      </c>
+      <c r="E11" s="14">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>213</v>
+      </c>
+      <c r="E12" s="14">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E90D8F56-706D-4721-87B3-B2321C52C97D}">
+  <dimension ref="A1:K36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="38" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="9" style="24" customWidth="1"/>
+    <col min="6" max="6" width="6" style="26" customWidth="1"/>
+    <col min="7" max="7" width="35" customWidth="1"/>
+    <col min="8" max="9" width="6" customWidth="1"/>
+    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="11" max="11" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="11" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="32">
+        <v>3</v>
+      </c>
+      <c r="G10" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="H10" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="K10" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="36" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" s="32">
+        <v>5</v>
+      </c>
+      <c r="G11" s="36" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I11" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J11" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="K11" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="31" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="D12" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" s="32">
+        <v>8</v>
+      </c>
+      <c r="G12" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I12" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J12" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="K12" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="31" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="D13" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" s="32">
+        <v>3</v>
+      </c>
+      <c r="G13" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="H13" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J13" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="K13" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B14" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="36" t="s">
+        <v>87</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="32">
+        <v>3</v>
+      </c>
+      <c r="G14" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I14" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J14" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="K14" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="32">
+        <v>3</v>
+      </c>
+      <c r="G15" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="H15" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I15" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J15" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="K15" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" s="32">
+        <v>3</v>
+      </c>
+      <c r="G16" s="36" t="s">
+        <v>96</v>
+      </c>
+      <c r="H16" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I16" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J16" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="K16" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="36" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F17" s="32">
+        <v>5</v>
+      </c>
+      <c r="G17" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I17" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J17" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="K17" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="36" t="s">
+        <v>103</v>
+      </c>
+      <c r="D18" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F18" s="32">
+        <v>5</v>
+      </c>
+      <c r="G18" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I18" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J18" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="K18" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="31" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="32">
+        <v>3</v>
+      </c>
+      <c r="G19" s="36" t="s">
+        <v>107</v>
+      </c>
+      <c r="H19" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I19" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J19" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="K19" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="36" t="s">
+        <v>110</v>
+      </c>
+      <c r="D20" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F20" s="32">
+        <v>5</v>
+      </c>
+      <c r="G20" s="42" t="s">
+        <v>111</v>
+      </c>
+      <c r="H20" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I20" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J20" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="K20" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="31" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="36" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F21" s="32">
+        <v>5</v>
+      </c>
+      <c r="G21" s="36" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I21" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J21" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="K21" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="31" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F22" s="32">
+        <v>5</v>
+      </c>
+      <c r="G22" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="H22" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I22" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J22" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="K22" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="B23" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="D23" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F23" s="32">
+        <v>8</v>
+      </c>
+      <c r="G23" s="36" t="s">
+        <v>123</v>
+      </c>
+      <c r="H23" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I23" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J23" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="K23" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="31" t="s">
+        <v>124</v>
+      </c>
+      <c r="B24" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="36" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E24" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F24" s="32">
+        <v>13</v>
+      </c>
+      <c r="G24" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="H24" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I24" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J24" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="K24" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="B25" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="36" t="s">
+        <v>129</v>
+      </c>
+      <c r="D25" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F25" s="32">
+        <v>8</v>
+      </c>
+      <c r="G25" s="36" t="s">
+        <v>130</v>
+      </c>
+      <c r="H25" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I25" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J25" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="K25" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="31" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" s="36" t="s">
+        <v>114</v>
+      </c>
+      <c r="E26" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F26" s="32">
+        <v>5</v>
+      </c>
+      <c r="G26" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="H26" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I26" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J26" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="K26" s="32" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="36" t="s">
+        <v>135</v>
+      </c>
+      <c r="D27" s="36" t="s">
+        <v>136</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="F27" s="32">
+        <v>13</v>
+      </c>
+      <c r="G27" s="36" t="s">
+        <v>138</v>
+      </c>
+      <c r="H27" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I27" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J27" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="K27" s="32" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="31" t="s">
+        <v>140</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C28" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="D28" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="F28" s="32">
+        <v>21</v>
+      </c>
+      <c r="G28" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="H28" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I28" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J28" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="K28" s="32" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="31" t="s">
+        <v>143</v>
+      </c>
+      <c r="B29" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="F29" s="32">
+        <v>13</v>
+      </c>
+      <c r="G29" s="36" t="s">
+        <v>145</v>
+      </c>
+      <c r="H29" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I29" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J29" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="K29" s="32" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="41" t="s">
+        <v>194</v>
+      </c>
+      <c r="B30" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="42" t="s">
+        <v>196</v>
+      </c>
+      <c r="D30" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="33">
+        <v>3</v>
+      </c>
+      <c r="G30" s="42" t="s">
+        <v>198</v>
+      </c>
+      <c r="H30" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I30" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J30" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="K30" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="41" t="s">
+        <v>195</v>
+      </c>
+      <c r="B31" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="42" t="s">
+        <v>197</v>
+      </c>
+      <c r="D31" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F31" s="33">
+        <v>4</v>
+      </c>
+      <c r="G31" s="42" t="s">
+        <v>199</v>
+      </c>
+      <c r="H31" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I31" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J31" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="K31" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="41" t="s">
+        <v>200</v>
+      </c>
+      <c r="B32" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="42" t="s">
+        <v>204</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F32" s="33">
+        <v>5</v>
+      </c>
+      <c r="G32" s="45" t="s">
+        <v>209</v>
+      </c>
+      <c r="H32" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I32" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J32" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="K32" s="46" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="41" t="s">
+        <v>201</v>
+      </c>
+      <c r="B33" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" s="42" t="s">
+        <v>207</v>
+      </c>
+      <c r="D33" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="F33" s="33">
+        <v>5</v>
+      </c>
+      <c r="G33" s="45" t="s">
+        <v>211</v>
+      </c>
+      <c r="H33" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I33" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J33" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="K33" s="46" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="41" t="s">
+        <v>202</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="42" t="s">
+        <v>205</v>
+      </c>
+      <c r="D34" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F34" s="33">
+        <v>3</v>
+      </c>
+      <c r="G34" s="45" t="s">
+        <v>212</v>
+      </c>
+      <c r="H34" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I34" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J34" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="K34" s="33" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="41" t="s">
+        <v>203</v>
+      </c>
+      <c r="B35" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="C35" s="42" t="s">
+        <v>206</v>
+      </c>
+      <c r="D35" s="36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="F35" s="33">
+        <v>4</v>
+      </c>
+      <c r="G35" s="42" t="s">
+        <v>210</v>
+      </c>
+      <c r="H35" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="I35" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="J35" s="33" t="s">
+        <v>108</v>
+      </c>
+      <c r="K35" s="46" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" s="37" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="38" t="s">
+        <v>146</v>
+      </c>
+      <c r="B36" s="35"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="35"/>
+      <c r="F36" s="34">
+        <f>SUM(F10:F35)</f>
+        <v>161</v>
+      </c>
+      <c r="G36" s="43" t="s">
+        <v>208</v>
+      </c>
+      <c r="H36" s="39"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="39"/>
+      <c r="K36" s="39"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Feuil5"/>
   <dimension ref="A1:A28"/>
@@ -2558,7 +3865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Feuil6"/>
   <dimension ref="A2:D15"/>
@@ -2678,7 +3985,7 @@
         <v>186</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="D15" s="23"/>
     </row>

</xml_diff>

<commit_message>
add perturbation recap caleb
</commit_message>
<xml_diff>
--- a/docs/cadrage/product-backlog.xlsx
+++ b/docs/cadrage/product-backlog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tsiba\Documents\cours\Master IA\apocalIPSSI\IPSSI_APOCAL_KIT_GR_28\docs\cadrage\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A47408-93F1-45EE-BE82-4D3FA25DE6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FF137F-24AB-401B-A8E6-18D55E695FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="25820" windowHeight="13900" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" r:id="rId1"/>
@@ -249,9 +249,6 @@
     <t>En tant qu'étudiant·e, je veux créer un compte avec email et mot de passe, afin de sauvegarder mes quizz et y revenir.</t>
   </si>
   <si>
-    <t>Étudiant·e</t>
-  </si>
-  <si>
     <t>MUST</t>
   </si>
   <si>
@@ -396,9 +393,6 @@
     <t>En tant qu'utilisateur·trice, je veux exporter toutes mes données en JSON et CSV, afin d'exercer mon droit d'accès Art. 15 RGPD.</t>
   </si>
   <si>
-    <t>Tous personas</t>
-  </si>
-  <si>
     <t>[1 critère type : bouton export → ZIP avec quizz.json + reponses.csv + audit.json]</t>
   </si>
   <si>
@@ -432,9 +426,6 @@
     <t>En tant qu'enseignant·e, je veux générer des questions ouvertes corrigées par le LLM, afin de varier les types d'évaluation.</t>
   </si>
   <si>
-    <t>Enseignant·e</t>
-  </si>
-  <si>
     <t>[1 critère type : mode 'question ouverte' avec barème indicatif et correction LLM]</t>
   </si>
   <si>
@@ -462,9 +453,6 @@
     <t>En tant que DSI d'établissement, je veux un SSO entreprise SAML/OIDC, afin d'intégrer EduTutor à mon AD/ENT.</t>
   </si>
   <si>
-    <t>Établissement</t>
-  </si>
-  <si>
     <t>WON'T</t>
   </si>
   <si>
@@ -619,9 +607,6 @@
   </si>
   <si>
     <t xml:space="preserve">Cadrage </t>
-  </si>
-  <si>
-    <t xml:space="preserve">v1.0 </t>
   </si>
   <si>
     <t xml:space="preserve">MAJ après perturbation </t>
@@ -745,6 +730,21 @@
   <si>
     <t>US-06, US-11, US-16,US-21
 US-22,US-23,US-25,US-26</t>
+  </si>
+  <si>
+    <t>Léa Martin</t>
+  </si>
+  <si>
+    <t>Mme Sophie Lefèvre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Léa Martin, Mme Sophie Lefèvre, David Chen </t>
+  </si>
+  <si>
+    <t xml:space="preserve">David Chen </t>
+  </si>
+  <si>
+    <t xml:space="preserve">v2.0 </t>
   </si>
 </sst>
 </file>
@@ -1531,7 +1531,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="27" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -1539,7 +1539,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -1547,7 +1547,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>189</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.35">
@@ -1563,7 +1563,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.35">
@@ -1841,698 +1841,698 @@
         <v>68</v>
       </c>
       <c r="D10" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E10" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F10" s="32">
         <v>3</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H10" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J10" s="32" t="s">
+      <c r="K10" s="32" t="s">
         <v>73</v>
-      </c>
-      <c r="K10" s="32" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B11" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E11" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F11" s="32">
         <v>5</v>
       </c>
       <c r="G11" s="36" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H11" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="I11" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" s="32" t="s">
+      <c r="K11" s="32" t="s">
         <v>73</v>
-      </c>
-      <c r="K11" s="32" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B12" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D12" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E12" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F12" s="32">
         <v>8</v>
       </c>
       <c r="G12" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H12" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I12" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J12" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J12" s="32" t="s">
-        <v>81</v>
-      </c>
       <c r="K12" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D13" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E13" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E13" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F13" s="32">
         <v>3</v>
       </c>
       <c r="G13" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="H13" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J13" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I13" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J13" s="32" t="s">
-        <v>85</v>
-      </c>
       <c r="K13" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="31" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D14" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E14" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E14" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F14" s="32">
         <v>3</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H14" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I14" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J14" s="32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K14" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B15" s="32" t="s">
         <v>42</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D15" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E15" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F15" s="32">
         <v>3</v>
       </c>
       <c r="G15" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J15" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="H15" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J15" s="32" t="s">
-        <v>92</v>
-      </c>
       <c r="K15" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B16" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>94</v>
-      </c>
-      <c r="D16" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>95</v>
       </c>
       <c r="F16" s="32">
         <v>3</v>
       </c>
       <c r="G16" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J16" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="H16" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I16" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J16" s="32" t="s">
+      <c r="K16" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K16" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="31" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B17" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D17" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F17" s="32">
         <v>5</v>
       </c>
       <c r="G17" s="36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H17" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I17" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J17" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="K17" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K17" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="31" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F18" s="32">
         <v>5</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H18" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I18" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J18" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="K18" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K18" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="31" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B19" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F19" s="32">
         <v>3</v>
       </c>
       <c r="G19" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I19" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J19" s="32" t="s">
         <v>107</v>
       </c>
-      <c r="H19" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I19" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J19" s="32" t="s">
-        <v>108</v>
-      </c>
       <c r="K19" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="32" t="s">
         <v>42</v>
       </c>
       <c r="C20" s="36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F20" s="32">
         <v>5</v>
       </c>
       <c r="G20" s="36" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H20" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I20" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J20" s="32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K20" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="31" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B21" s="32" t="s">
         <v>46</v>
       </c>
       <c r="C21" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D21" s="36" t="s">
-        <v>114</v>
+        <v>212</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F21" s="32">
         <v>5</v>
       </c>
       <c r="G21" s="36" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I21" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J21" s="32" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="K21" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="31" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B22" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C22" s="36" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F22" s="32">
         <v>5</v>
       </c>
       <c r="G22" s="36" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H22" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I22" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J22" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="I22" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J22" s="33" t="s">
-        <v>73</v>
-      </c>
       <c r="K22" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="31" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B23" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="36" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F23" s="32">
         <v>8</v>
       </c>
       <c r="G23" s="36" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I23" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J23" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="K23" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K23" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B24" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F24" s="32">
         <v>13</v>
       </c>
       <c r="G24" s="36" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H24" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I24" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J24" s="33" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K24" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="31" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B25" s="32" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D25" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F25" s="32">
         <v>8</v>
       </c>
       <c r="G25" s="36" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H25" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I25" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J25" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K25" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="31" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B26" s="32" t="s">
         <v>46</v>
       </c>
       <c r="C26" s="36" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>114</v>
+        <v>212</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F26" s="32">
         <v>5</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H26" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I26" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J26" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="I26" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J26" s="33" t="s">
-        <v>73</v>
-      </c>
       <c r="K26" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="31" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B27" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C27" s="36" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>136</v>
+        <v>213</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F27" s="32">
         <v>13</v>
       </c>
       <c r="G27" s="36" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H27" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I27" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J27" s="33" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K27" s="32" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="31" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B28" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F28" s="32">
         <v>21</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="H28" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I28" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J28" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K28" s="32" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="31" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B29" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C29" s="36" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E29" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F29" s="32">
         <v>13</v>
       </c>
       <c r="G29" s="36" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="H29" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I29" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J29" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K29" s="32" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" spans="1:11" s="37" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="38" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B30" s="35"/>
       <c r="C30" s="39"/>
@@ -2542,7 +2542,7 @@
         <v>137</v>
       </c>
       <c r="G30" s="40" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="H30" s="39"/>
       <c r="I30" s="39"/>
@@ -2680,7 +2680,7 @@
         <v>44</v>
       </c>
       <c r="D11" s="44" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E11" s="14">
         <v>35</v>
@@ -2697,7 +2697,7 @@
         <v>48</v>
       </c>
       <c r="D12" s="44" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="E12" s="14">
         <v>15</v>
@@ -2812,908 +2812,908 @@
         <v>68</v>
       </c>
       <c r="D10" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E10" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F10" s="32">
         <v>3</v>
       </c>
       <c r="G10" s="36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H10" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J10" s="32" t="s">
+      <c r="K10" s="32" t="s">
         <v>73</v>
-      </c>
-      <c r="K10" s="32" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B11" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D11" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E11" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F11" s="32">
         <v>5</v>
       </c>
       <c r="G11" s="36" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H11" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J11" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="I11" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" s="32" t="s">
+      <c r="K11" s="32" t="s">
         <v>73</v>
-      </c>
-      <c r="K11" s="32" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B12" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="36" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D12" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E12" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F12" s="32">
         <v>8</v>
       </c>
       <c r="G12" s="36" t="s">
+        <v>79</v>
+      </c>
+      <c r="H12" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I12" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J12" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J12" s="32" t="s">
-        <v>81</v>
-      </c>
       <c r="K12" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D13" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E13" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E13" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F13" s="32">
         <v>3</v>
       </c>
       <c r="G13" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="H13" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J13" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I13" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J13" s="32" t="s">
-        <v>85</v>
-      </c>
       <c r="K13" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="31" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D14" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E14" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E14" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F14" s="32">
         <v>3</v>
       </c>
       <c r="G14" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H14" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I14" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J14" s="32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K14" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="31" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B15" s="32" t="s">
         <v>42</v>
       </c>
       <c r="C15" s="36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D15" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E15" s="17" t="s">
         <v>69</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="F15" s="32">
         <v>3</v>
       </c>
       <c r="G15" s="42" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J15" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="H15" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J15" s="32" t="s">
-        <v>92</v>
-      </c>
       <c r="K15" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B16" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>210</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>94</v>
-      </c>
-      <c r="D16" s="36" t="s">
-        <v>69</v>
-      </c>
-      <c r="E16" s="18" t="s">
-        <v>95</v>
       </c>
       <c r="F16" s="32">
         <v>3</v>
       </c>
       <c r="G16" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J16" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="H16" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I16" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J16" s="32" t="s">
+      <c r="K16" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K16" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="31" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B17" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="36" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D17" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F17" s="32">
         <v>5</v>
       </c>
       <c r="G17" s="36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H17" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I17" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J17" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="K17" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K17" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="31" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C18" s="36" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D18" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F18" s="32">
         <v>5</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H18" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I18" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J18" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="K18" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K18" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="31" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B19" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C19" s="36" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D19" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F19" s="32">
         <v>3</v>
       </c>
       <c r="G19" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I19" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J19" s="32" t="s">
         <v>107</v>
       </c>
-      <c r="H19" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="I19" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J19" s="32" t="s">
-        <v>108</v>
-      </c>
       <c r="K19" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B20" s="32" t="s">
         <v>42</v>
       </c>
       <c r="C20" s="36" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F20" s="32">
         <v>5</v>
       </c>
       <c r="G20" s="42" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H20" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I20" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J20" s="32" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K20" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="31" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B21" s="32" t="s">
         <v>46</v>
       </c>
       <c r="C21" s="36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D21" s="36" t="s">
-        <v>114</v>
+        <v>212</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F21" s="32">
         <v>5</v>
       </c>
       <c r="G21" s="36" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H21" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I21" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J21" s="32" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="K21" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="31" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B22" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C22" s="36" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D22" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F22" s="32">
         <v>5</v>
       </c>
       <c r="G22" s="36" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H22" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I22" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J22" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="I22" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J22" s="33" t="s">
-        <v>73</v>
-      </c>
       <c r="K22" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="31" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B23" s="32" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="36" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D23" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E23" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F23" s="32">
         <v>8</v>
       </c>
       <c r="G23" s="36" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H23" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I23" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J23" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="K23" s="32" t="s">
         <v>97</v>
-      </c>
-      <c r="K23" s="32" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B24" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C24" s="36" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D24" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F24" s="32">
         <v>13</v>
       </c>
       <c r="G24" s="36" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H24" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I24" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J24" s="33" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K24" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="31" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B25" s="32" t="s">
         <v>42</v>
       </c>
       <c r="C25" s="36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D25" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F25" s="32">
         <v>8</v>
       </c>
       <c r="G25" s="36" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H25" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I25" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J25" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K25" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="31" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B26" s="32" t="s">
         <v>46</v>
       </c>
       <c r="C26" s="36" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>114</v>
+        <v>212</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F26" s="32">
         <v>5</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="H26" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I26" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="J26" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="I26" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="J26" s="33" t="s">
-        <v>73</v>
-      </c>
       <c r="K26" s="32" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="27" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="31" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B27" s="32" t="s">
         <v>26</v>
       </c>
       <c r="C27" s="36" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D27" s="36" t="s">
-        <v>136</v>
+        <v>213</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F27" s="32">
         <v>13</v>
       </c>
       <c r="G27" s="36" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H27" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I27" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J27" s="33" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K27" s="32" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="31" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B28" s="32" t="s">
         <v>34</v>
       </c>
       <c r="C28" s="36" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F28" s="32">
         <v>21</v>
       </c>
       <c r="G28" s="36" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="H28" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I28" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J28" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K28" s="32" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="31" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B29" s="32" t="s">
         <v>38</v>
       </c>
       <c r="C29" s="36" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D29" s="36" t="s">
-        <v>69</v>
+        <v>210</v>
       </c>
       <c r="E29" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F29" s="32">
         <v>13</v>
       </c>
       <c r="G29" s="36" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="H29" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I29" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J29" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K29" s="32" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="41" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B30" s="33" t="s">
         <v>42</v>
       </c>
       <c r="C30" s="42" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D30" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F30" s="33">
         <v>3</v>
       </c>
       <c r="G30" s="42" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="H30" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I30" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J30" s="32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K30" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="41" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B31" s="33" t="s">
         <v>42</v>
       </c>
       <c r="C31" s="42" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="D31" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F31" s="33">
         <v>4</v>
       </c>
       <c r="G31" s="42" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="H31" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I31" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J31" s="32" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K31" s="32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="32" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="41" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B32" s="33" t="s">
         <v>42</v>
       </c>
       <c r="C32" s="42" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="D32" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F32" s="33">
         <v>5</v>
       </c>
       <c r="G32" s="45" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="H32" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I32" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J32" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K32" s="46" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="33" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="41" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B33" s="33" t="s">
         <v>46</v>
       </c>
       <c r="C33" s="42" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="D33" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E33" s="18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F33" s="33">
         <v>5</v>
       </c>
       <c r="G33" s="45" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="H33" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I33" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J33" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K33" s="46" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="41" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B34" s="33" t="s">
         <v>42</v>
       </c>
       <c r="C34" s="42" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D34" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F34" s="33">
         <v>3</v>
       </c>
       <c r="G34" s="45" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="H34" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I34" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J34" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K34" s="33" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:11" s="37" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="41" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B35" s="33" t="s">
         <v>42</v>
       </c>
       <c r="C35" s="42" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D35" s="36" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F35" s="33">
         <v>4</v>
       </c>
       <c r="G35" s="42" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="H35" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I35" s="32" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J35" s="33" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K35" s="46" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="36" spans="1:11" s="37" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="38" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B36" s="35"/>
       <c r="C36" s="39"/>
@@ -3724,7 +3724,7 @@
         <v>161</v>
       </c>
       <c r="G36" s="43" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="H36" s="39"/>
       <c r="I36" s="39"/>
@@ -3747,117 +3747,117 @@
   <sheetData>
     <row r="1" spans="1:1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="11" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A4" s="21" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="22" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="22" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" s="22" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" s="22" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" s="22" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" s="22" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" s="22" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" s="22" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A17" s="21" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="9" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="22" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" s="22" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" s="22" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" s="22" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" s="22" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" s="22" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" s="22" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" s="22" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -3879,113 +3879,113 @@
   <sheetData>
     <row r="2" spans="1:4" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B2" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B3" s="9" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="12"/>
       <c r="B5" s="12" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D5" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="23" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D6" s="23"/>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="23" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D7" s="23"/>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="23" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D8" s="23"/>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="23" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D9" s="23"/>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="23" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D10" s="23"/>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="23" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D11" s="23"/>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="23" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D12" s="23"/>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="23" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="D13" s="23"/>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="23" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D14" s="23"/>
     </row>
     <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="C15" s="24" t="s">
         <v>186</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>191</v>
       </c>
       <c r="D15" s="23"/>
     </row>

</xml_diff>